<commit_message>
se incorpora algunas metricas
</commit_message>
<xml_diff>
--- a/output/comentarios_procesados.xlsx
+++ b/output/comentarios_procesados.xlsx
@@ -481,7 +481,7 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -497,7 +497,7 @@
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -513,7 +513,7 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -529,7 +529,7 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -561,7 +561,7 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -577,7 +577,7 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="10">
@@ -593,7 +593,7 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -609,7 +609,7 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="12">
@@ -641,7 +641,7 @@
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -657,7 +657,7 @@
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="15">
@@ -673,7 +673,7 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -705,7 +705,7 @@
         <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -737,7 +737,7 @@
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -753,7 +753,7 @@
         <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -769,7 +769,7 @@
         <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="22">
@@ -785,7 +785,7 @@
         <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="23">
@@ -801,7 +801,7 @@
         <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -833,7 +833,7 @@
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -849,7 +849,7 @@
         <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="27">
@@ -881,7 +881,7 @@
         <v>1</v>
       </c>
       <c r="D28" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -897,7 +897,7 @@
         <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="30">
@@ -961,7 +961,7 @@
         <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -977,7 +977,7 @@
         <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -993,7 +993,7 @@
         <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -1041,7 +1041,7 @@
         <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -1073,7 +1073,7 @@
         <v>1</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="41">
@@ -1121,7 +1121,7 @@
         <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -1169,7 +1169,7 @@
         <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="47">
@@ -1185,7 +1185,7 @@
         <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -1201,7 +1201,7 @@
         <v>1</v>
       </c>
       <c r="D48" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -1217,7 +1217,7 @@
         <v>1</v>
       </c>
       <c r="D49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -1233,7 +1233,7 @@
         <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="51">
@@ -1265,7 +1265,7 @@
         <v>1</v>
       </c>
       <c r="D52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -1281,7 +1281,7 @@
         <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="54">
@@ -1297,7 +1297,7 @@
         <v>1</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -1313,7 +1313,7 @@
         <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -1345,7 +1345,7 @@
         <v>1</v>
       </c>
       <c r="D57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -1361,7 +1361,7 @@
         <v>1</v>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="59">
@@ -1377,7 +1377,7 @@
         <v>1</v>
       </c>
       <c r="D59" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="60">
@@ -1393,7 +1393,7 @@
         <v>1</v>
       </c>
       <c r="D60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -1457,7 +1457,7 @@
         <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -1505,7 +1505,7 @@
         <v>1</v>
       </c>
       <c r="D67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -1537,7 +1537,7 @@
         <v>1</v>
       </c>
       <c r="D69" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="70">
@@ -1553,7 +1553,7 @@
         <v>1</v>
       </c>
       <c r="D70" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -1569,7 +1569,7 @@
         <v>1</v>
       </c>
       <c r="D71" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -1601,7 +1601,7 @@
         <v>1</v>
       </c>
       <c r="D73" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -1617,7 +1617,7 @@
         <v>1</v>
       </c>
       <c r="D74" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="75">
@@ -1633,7 +1633,7 @@
         <v>1</v>
       </c>
       <c r="D75" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -1665,7 +1665,7 @@
         <v>1</v>
       </c>
       <c r="D77" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -1697,7 +1697,7 @@
         <v>1</v>
       </c>
       <c r="D79" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -1713,7 +1713,7 @@
         <v>1</v>
       </c>
       <c r="D80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81">
@@ -1729,7 +1729,7 @@
         <v>1</v>
       </c>
       <c r="D81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -1745,7 +1745,7 @@
         <v>1</v>
       </c>
       <c r="D82" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -1777,7 +1777,7 @@
         <v>1</v>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -1793,7 +1793,7 @@
         <v>1</v>
       </c>
       <c r="D85" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="86">
@@ -1809,7 +1809,7 @@
         <v>1</v>
       </c>
       <c r="D86" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87">
@@ -1873,7 +1873,7 @@
         <v>1</v>
       </c>
       <c r="D90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91">
@@ -1889,7 +1889,7 @@
         <v>1</v>
       </c>
       <c r="D91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -1905,7 +1905,7 @@
         <v>1</v>
       </c>
       <c r="D92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -1921,7 +1921,7 @@
         <v>1</v>
       </c>
       <c r="D93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -1937,7 +1937,7 @@
         <v>1</v>
       </c>
       <c r="D94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95">
@@ -1953,7 +1953,7 @@
         <v>1</v>
       </c>
       <c r="D95" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -1985,7 +1985,7 @@
         <v>1</v>
       </c>
       <c r="D97" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
@@ -2001,7 +2001,7 @@
         <v>1</v>
       </c>
       <c r="D98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99">
@@ -2017,7 +2017,7 @@
         <v>1</v>
       </c>
       <c r="D99" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -2033,7 +2033,7 @@
         <v>1</v>
       </c>
       <c r="D100" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="101">
@@ -2049,7 +2049,7 @@
         <v>1</v>
       </c>
       <c r="D101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102">
@@ -2065,7 +2065,7 @@
         <v>1</v>
       </c>
       <c r="D102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -2081,7 +2081,7 @@
         <v>1</v>
       </c>
       <c r="D103" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104">
@@ -2097,7 +2097,7 @@
         <v>1</v>
       </c>
       <c r="D104" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105">
@@ -2129,7 +2129,7 @@
         <v>1</v>
       </c>
       <c r="D106" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
@@ -2161,7 +2161,7 @@
         <v>1</v>
       </c>
       <c r="D108" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -2209,7 +2209,7 @@
         <v>1</v>
       </c>
       <c r="D111" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112">
@@ -2225,7 +2225,7 @@
         <v>1</v>
       </c>
       <c r="D112" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="113">
@@ -2257,7 +2257,7 @@
         <v>1</v>
       </c>
       <c r="D114" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="115">
@@ -2273,7 +2273,7 @@
         <v>1</v>
       </c>
       <c r="D115" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116">
@@ -2289,7 +2289,7 @@
         <v>1</v>
       </c>
       <c r="D116" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="117">
@@ -2305,7 +2305,7 @@
         <v>1</v>
       </c>
       <c r="D117" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="118">
@@ -2321,7 +2321,7 @@
         <v>1</v>
       </c>
       <c r="D118" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119">
@@ -2337,7 +2337,7 @@
         <v>1</v>
       </c>
       <c r="D119" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120">
@@ -2353,7 +2353,7 @@
         <v>1</v>
       </c>
       <c r="D120" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="121">
@@ -2385,7 +2385,7 @@
         <v>1</v>
       </c>
       <c r="D122" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="123">
@@ -2401,7 +2401,7 @@
         <v>1</v>
       </c>
       <c r="D123" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124">
@@ -2417,7 +2417,7 @@
         <v>1</v>
       </c>
       <c r="D124" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="125">
@@ -2465,7 +2465,7 @@
         <v>1</v>
       </c>
       <c r="D127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="128">
@@ -2497,7 +2497,7 @@
         <v>1</v>
       </c>
       <c r="D129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130">
@@ -2513,7 +2513,7 @@
         <v>1</v>
       </c>
       <c r="D130" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="131">
@@ -2529,7 +2529,7 @@
         <v>1</v>
       </c>
       <c r="D131" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132">
@@ -2545,7 +2545,7 @@
         <v>1</v>
       </c>
       <c r="D132" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="133">
@@ -2561,7 +2561,7 @@
         <v>1</v>
       </c>
       <c r="D133" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134">
@@ -2577,7 +2577,7 @@
         <v>1</v>
       </c>
       <c r="D134" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="135">
@@ -2593,7 +2593,7 @@
         <v>1</v>
       </c>
       <c r="D135" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="136">
@@ -2657,7 +2657,7 @@
         <v>1</v>
       </c>
       <c r="D139" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="140">
@@ -2673,7 +2673,7 @@
         <v>1</v>
       </c>
       <c r="D140" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="141">
@@ -2705,7 +2705,7 @@
         <v>1</v>
       </c>
       <c r="D142" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="143">
@@ -2753,7 +2753,7 @@
         <v>1</v>
       </c>
       <c r="D145" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146">
@@ -2769,7 +2769,7 @@
         <v>1</v>
       </c>
       <c r="D146" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="147">
@@ -2817,7 +2817,7 @@
         <v>1</v>
       </c>
       <c r="D149" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="150">
@@ -2849,7 +2849,7 @@
         <v>1</v>
       </c>
       <c r="D151" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152">
@@ -2865,7 +2865,7 @@
         <v>1</v>
       </c>
       <c r="D152" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="153">
@@ -2897,7 +2897,7 @@
         <v>1</v>
       </c>
       <c r="D154" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="155">
@@ -2929,7 +2929,7 @@
         <v>1</v>
       </c>
       <c r="D156" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="157">
@@ -3025,7 +3025,7 @@
         <v>1</v>
       </c>
       <c r="D162" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="163">
@@ -3041,7 +3041,7 @@
         <v>1</v>
       </c>
       <c r="D163" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="164">
@@ -3057,7 +3057,7 @@
         <v>1</v>
       </c>
       <c r="D164" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="165">
@@ -3089,7 +3089,7 @@
         <v>1</v>
       </c>
       <c r="D166" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167">
@@ -3105,7 +3105,7 @@
         <v>1</v>
       </c>
       <c r="D167" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168">
@@ -3121,7 +3121,7 @@
         <v>1</v>
       </c>
       <c r="D168" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="169">
@@ -3137,7 +3137,7 @@
         <v>1</v>
       </c>
       <c r="D169" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="170">
@@ -3153,7 +3153,7 @@
         <v>1</v>
       </c>
       <c r="D170" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="171">
@@ -3169,7 +3169,7 @@
         <v>1</v>
       </c>
       <c r="D171" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="172">
@@ -3185,7 +3185,7 @@
         <v>1</v>
       </c>
       <c r="D172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173">
@@ -3201,7 +3201,7 @@
         <v>1</v>
       </c>
       <c r="D173" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="174">
@@ -3249,7 +3249,7 @@
         <v>1</v>
       </c>
       <c r="D176" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177">
@@ -3265,7 +3265,7 @@
         <v>1</v>
       </c>
       <c r="D177" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178">
@@ -3297,7 +3297,7 @@
         <v>1</v>
       </c>
       <c r="D179" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="180">
@@ -3313,7 +3313,7 @@
         <v>1</v>
       </c>
       <c r="D180" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="181">
@@ -3345,7 +3345,7 @@
         <v>1</v>
       </c>
       <c r="D182" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="183">
@@ -3377,7 +3377,7 @@
         <v>1</v>
       </c>
       <c r="D184" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="185">
@@ -3393,7 +3393,7 @@
         <v>1</v>
       </c>
       <c r="D185" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="186">
@@ -3409,7 +3409,7 @@
         <v>1</v>
       </c>
       <c r="D186" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="187">
@@ -3441,7 +3441,7 @@
         <v>1</v>
       </c>
       <c r="D188" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="189">
@@ -3457,7 +3457,7 @@
         <v>1</v>
       </c>
       <c r="D189" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="190">
@@ -3473,7 +3473,7 @@
         <v>1</v>
       </c>
       <c r="D190" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="191">
@@ -3489,7 +3489,7 @@
         <v>1</v>
       </c>
       <c r="D191" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="192">
@@ -3521,7 +3521,7 @@
         <v>1</v>
       </c>
       <c r="D193" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="194">
@@ -3537,7 +3537,7 @@
         <v>1</v>
       </c>
       <c r="D194" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="195">
@@ -3553,7 +3553,7 @@
         <v>1</v>
       </c>
       <c r="D195" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="196">
@@ -3569,7 +3569,7 @@
         <v>1</v>
       </c>
       <c r="D196" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="197">
@@ -3585,7 +3585,7 @@
         <v>1</v>
       </c>
       <c r="D197" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198">
@@ -3617,7 +3617,7 @@
         <v>1</v>
       </c>
       <c r="D199" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="200">
@@ -3633,7 +3633,7 @@
         <v>1</v>
       </c>
       <c r="D200" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="201">
@@ -3701,7 +3701,7 @@
         <v>-1</v>
       </c>
       <c r="D2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -3765,7 +3765,7 @@
         <v>-1</v>
       </c>
       <c r="D6" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -3781,7 +3781,7 @@
         <v>-1</v>
       </c>
       <c r="D7" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -3797,7 +3797,7 @@
         <v>-1</v>
       </c>
       <c r="D8" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -3813,7 +3813,7 @@
         <v>-1</v>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="10">
@@ -3845,7 +3845,7 @@
         <v>-1</v>
       </c>
       <c r="D11" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -3861,7 +3861,7 @@
         <v>-1</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="13">
@@ -3893,7 +3893,7 @@
         <v>-1</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="15">
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="D15" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -3925,7 +3925,7 @@
         <v>-1</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="17">
@@ -3957,7 +3957,7 @@
         <v>-1</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="19">
@@ -3973,7 +3973,7 @@
         <v>-1</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -3989,7 +3989,7 @@
         <v>-1</v>
       </c>
       <c r="D20" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -4005,7 +4005,7 @@
         <v>-1</v>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="22">
@@ -4037,7 +4037,7 @@
         <v>-1</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="24">
@@ -4069,7 +4069,7 @@
         <v>-1</v>
       </c>
       <c r="D25" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -4085,7 +4085,7 @@
         <v>-1</v>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="27">
@@ -4101,7 +4101,7 @@
         <v>-1</v>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="28">
@@ -4117,7 +4117,7 @@
         <v>-1</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="29">
@@ -4133,7 +4133,7 @@
         <v>-1</v>
       </c>
       <c r="D29" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -4149,7 +4149,7 @@
         <v>-1</v>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -4165,7 +4165,7 @@
         <v>-1</v>
       </c>
       <c r="D31" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -4181,7 +4181,7 @@
         <v>-1</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -4197,7 +4197,7 @@
         <v>-1</v>
       </c>
       <c r="D33" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -4213,7 +4213,7 @@
         <v>-1</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -4229,7 +4229,7 @@
         <v>-1</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -4245,7 +4245,7 @@
         <v>-1</v>
       </c>
       <c r="D36" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -4277,7 +4277,7 @@
         <v>-1</v>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="39">
@@ -4293,7 +4293,7 @@
         <v>-1</v>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="40">
@@ -4309,7 +4309,7 @@
         <v>-1</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="41">
@@ -4357,7 +4357,7 @@
         <v>-1</v>
       </c>
       <c r="D43" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -4373,7 +4373,7 @@
         <v>-1</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -4389,7 +4389,7 @@
         <v>-1</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="46">
@@ -4405,7 +4405,7 @@
         <v>-1</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="47">
@@ -4421,7 +4421,7 @@
         <v>-1</v>
       </c>
       <c r="D47" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -4485,7 +4485,7 @@
         <v>-1</v>
       </c>
       <c r="D51" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -4501,7 +4501,7 @@
         <v>-1</v>
       </c>
       <c r="D52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -4517,7 +4517,7 @@
         <v>-1</v>
       </c>
       <c r="D53" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -4533,7 +4533,7 @@
         <v>-1</v>
       </c>
       <c r="D54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -4549,7 +4549,7 @@
         <v>-1</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -4597,7 +4597,7 @@
         <v>-1</v>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="59">
@@ -4613,7 +4613,7 @@
         <v>-1</v>
       </c>
       <c r="D59" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="60">
@@ -4629,7 +4629,7 @@
         <v>-1</v>
       </c>
       <c r="D60" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="61">
@@ -4645,7 +4645,7 @@
         <v>-1</v>
       </c>
       <c r="D61" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -4661,7 +4661,7 @@
         <v>-1</v>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="63">
@@ -4693,7 +4693,7 @@
         <v>-1</v>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="65">
@@ -4709,7 +4709,7 @@
         <v>-1</v>
       </c>
       <c r="D65" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -4725,7 +4725,7 @@
         <v>-1</v>
       </c>
       <c r="D66" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -4741,7 +4741,7 @@
         <v>-1</v>
       </c>
       <c r="D67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="D68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -4773,7 +4773,7 @@
         <v>-1</v>
       </c>
       <c r="D69" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -4789,7 +4789,7 @@
         <v>-1</v>
       </c>
       <c r="D70" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="71">
@@ -4805,7 +4805,7 @@
         <v>-1</v>
       </c>
       <c r="D71" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="72">
@@ -4821,7 +4821,7 @@
         <v>-1</v>
       </c>
       <c r="D72" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -4853,7 +4853,7 @@
         <v>-1</v>
       </c>
       <c r="D74" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -4869,7 +4869,7 @@
         <v>-1</v>
       </c>
       <c r="D75" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -4917,7 +4917,7 @@
         <v>-1</v>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -4949,7 +4949,7 @@
         <v>-1</v>
       </c>
       <c r="D80" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="81">
@@ -4981,7 +4981,7 @@
         <v>-1</v>
       </c>
       <c r="D82" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -5013,7 +5013,7 @@
         <v>-1</v>
       </c>
       <c r="D84" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85">
@@ -5029,7 +5029,7 @@
         <v>-1</v>
       </c>
       <c r="D85" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -5045,7 +5045,7 @@
         <v>-1</v>
       </c>
       <c r="D86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87">
@@ -5061,7 +5061,7 @@
         <v>-1</v>
       </c>
       <c r="D87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -5109,7 +5109,7 @@
         <v>-1</v>
       </c>
       <c r="D90" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91">
@@ -5141,7 +5141,7 @@
         <v>-1</v>
       </c>
       <c r="D92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -5205,7 +5205,7 @@
         <v>-1</v>
       </c>
       <c r="D96" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="97">
@@ -5221,7 +5221,7 @@
         <v>-1</v>
       </c>
       <c r="D97" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
@@ -5237,7 +5237,7 @@
         <v>-1</v>
       </c>
       <c r="D98" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99">
@@ -5253,7 +5253,7 @@
         <v>-1</v>
       </c>
       <c r="D99" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100">
@@ -5301,7 +5301,7 @@
         <v>-1</v>
       </c>
       <c r="D102" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -5349,7 +5349,7 @@
         <v>-1</v>
       </c>
       <c r="D105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
@@ -5397,7 +5397,7 @@
         <v>-1</v>
       </c>
       <c r="D108" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="109">
@@ -5445,7 +5445,7 @@
         <v>-1</v>
       </c>
       <c r="D111" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="112">
@@ -5461,7 +5461,7 @@
         <v>-1</v>
       </c>
       <c r="D112" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -5477,7 +5477,7 @@
         <v>-1</v>
       </c>
       <c r="D113" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114">
@@ -5493,7 +5493,7 @@
         <v>-1</v>
       </c>
       <c r="D114" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115">
@@ -5525,7 +5525,7 @@
         <v>-1</v>
       </c>
       <c r="D116" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="117">
@@ -5541,7 +5541,7 @@
         <v>-1</v>
       </c>
       <c r="D117" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118">
@@ -5557,7 +5557,7 @@
         <v>-1</v>
       </c>
       <c r="D118" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="119">
@@ -5573,7 +5573,7 @@
         <v>-1</v>
       </c>
       <c r="D119" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120">
@@ -5589,7 +5589,7 @@
         <v>-1</v>
       </c>
       <c r="D120" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="121">
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="D121" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122">
@@ -5637,7 +5637,7 @@
         <v>-1</v>
       </c>
       <c r="D123" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="124">
@@ -5685,7 +5685,7 @@
         <v>-1</v>
       </c>
       <c r="D126" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="127">
@@ -5701,7 +5701,7 @@
         <v>-1</v>
       </c>
       <c r="D127" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="128">
@@ -5717,7 +5717,7 @@
         <v>-1</v>
       </c>
       <c r="D128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129">
@@ -5733,7 +5733,7 @@
         <v>-1</v>
       </c>
       <c r="D129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130">
@@ -5749,7 +5749,7 @@
         <v>-1</v>
       </c>
       <c r="D130" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="131">
@@ -5797,7 +5797,7 @@
         <v>-1</v>
       </c>
       <c r="D133" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134">
@@ -5829,7 +5829,7 @@
         <v>-1</v>
       </c>
       <c r="D135" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136">
@@ -5845,7 +5845,7 @@
         <v>-1</v>
       </c>
       <c r="D136" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="137">
@@ -5877,7 +5877,7 @@
         <v>-1</v>
       </c>
       <c r="D138" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139">
@@ -5925,7 +5925,7 @@
         <v>-1</v>
       </c>
       <c r="D141" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="142">
@@ -5941,7 +5941,7 @@
         <v>-1</v>
       </c>
       <c r="D142" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143">
@@ -5957,7 +5957,7 @@
         <v>-1</v>
       </c>
       <c r="D143" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="144">
@@ -5973,7 +5973,7 @@
         <v>-1</v>
       </c>
       <c r="D144" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145">
@@ -5989,7 +5989,7 @@
         <v>-1</v>
       </c>
       <c r="D145" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146">
@@ -6005,7 +6005,7 @@
         <v>-1</v>
       </c>
       <c r="D146" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="147">
@@ -6037,7 +6037,7 @@
         <v>-1</v>
       </c>
       <c r="D148" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149">
@@ -6053,7 +6053,7 @@
         <v>-1</v>
       </c>
       <c r="D149" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="150">
@@ -6069,7 +6069,7 @@
         <v>-1</v>
       </c>
       <c r="D150" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="151">
@@ -6085,7 +6085,7 @@
         <v>-1</v>
       </c>
       <c r="D151" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152">
@@ -6101,7 +6101,7 @@
         <v>-1</v>
       </c>
       <c r="D152" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="153">
@@ -6117,7 +6117,7 @@
         <v>-1</v>
       </c>
       <c r="D153" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="154">
@@ -6149,7 +6149,7 @@
         <v>-1</v>
       </c>
       <c r="D155" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156">
@@ -6165,7 +6165,7 @@
         <v>-1</v>
       </c>
       <c r="D156" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="157">
@@ -6181,7 +6181,7 @@
         <v>-1</v>
       </c>
       <c r="D157" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="158">
@@ -6197,7 +6197,7 @@
         <v>-1</v>
       </c>
       <c r="D158" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="159">
@@ -6229,7 +6229,7 @@
         <v>-1</v>
       </c>
       <c r="D160" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="161">
@@ -6277,7 +6277,7 @@
         <v>-1</v>
       </c>
       <c r="D163" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="164">
@@ -6293,7 +6293,7 @@
         <v>-1</v>
       </c>
       <c r="D164" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="165">
@@ -6309,7 +6309,7 @@
         <v>-1</v>
       </c>
       <c r="D165" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="166">
@@ -6325,7 +6325,7 @@
         <v>-1</v>
       </c>
       <c r="D166" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="167">
@@ -6357,7 +6357,7 @@
         <v>-1</v>
       </c>
       <c r="D168" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="169">
@@ -6373,7 +6373,7 @@
         <v>-1</v>
       </c>
       <c r="D169" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="170">
@@ -6389,7 +6389,7 @@
         <v>-1</v>
       </c>
       <c r="D170" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="171">
@@ -6405,7 +6405,7 @@
         <v>-1</v>
       </c>
       <c r="D171" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="172">
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="D174" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="175">
@@ -6485,7 +6485,7 @@
         <v>-1</v>
       </c>
       <c r="D176" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="177">
@@ -6501,7 +6501,7 @@
         <v>-1</v>
       </c>
       <c r="D177" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178">
@@ -6533,7 +6533,7 @@
         <v>-1</v>
       </c>
       <c r="D179" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="180">
@@ -6645,7 +6645,7 @@
         <v>-1</v>
       </c>
       <c r="D186" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="187">
@@ -6677,7 +6677,7 @@
         <v>-1</v>
       </c>
       <c r="D188" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="189">
@@ -6693,7 +6693,7 @@
         <v>-1</v>
       </c>
       <c r="D189" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="190">
@@ -6709,7 +6709,7 @@
         <v>-1</v>
       </c>
       <c r="D190" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="191">
@@ -6741,7 +6741,7 @@
         <v>-1</v>
       </c>
       <c r="D192" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193">
@@ -6757,7 +6757,7 @@
         <v>-1</v>
       </c>
       <c r="D193" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="194">
@@ -6773,7 +6773,7 @@
         <v>-1</v>
       </c>
       <c r="D194" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="195">
@@ -6789,7 +6789,7 @@
         <v>-1</v>
       </c>
       <c r="D195" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="196">
@@ -6805,7 +6805,7 @@
         <v>-1</v>
       </c>
       <c r="D196" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="197">
@@ -6837,7 +6837,7 @@
         <v>-1</v>
       </c>
       <c r="D198" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199">
@@ -6937,7 +6937,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -6953,7 +6953,7 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -6969,7 +6969,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -6985,7 +6985,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -7001,7 +7001,7 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -7017,7 +7017,7 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -7065,7 +7065,7 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -7081,7 +7081,7 @@
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -7097,7 +7097,7 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -7113,7 +7113,7 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -7129,7 +7129,7 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -7145,7 +7145,7 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="16">
@@ -7161,7 +7161,7 @@
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -7177,7 +7177,7 @@
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="18">
@@ -7193,7 +7193,7 @@
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="19">
@@ -7209,7 +7209,7 @@
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -7225,7 +7225,7 @@
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="21">
@@ -7241,7 +7241,7 @@
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="22">
@@ -7257,7 +7257,7 @@
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -7273,7 +7273,7 @@
         <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -7289,7 +7289,7 @@
         <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="25">
@@ -7305,7 +7305,7 @@
         <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="26">
@@ -7337,7 +7337,7 @@
         <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -7385,7 +7385,7 @@
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="31">
@@ -7401,7 +7401,7 @@
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -7417,7 +7417,7 @@
         <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -7433,7 +7433,7 @@
         <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -7449,7 +7449,7 @@
         <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -7465,7 +7465,7 @@
         <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="36">
@@ -7481,7 +7481,7 @@
         <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -7513,7 +7513,7 @@
         <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -7545,7 +7545,7 @@
         <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -7561,7 +7561,7 @@
         <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="42">
@@ -7577,7 +7577,7 @@
         <v>0</v>
       </c>
       <c r="D42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -7593,7 +7593,7 @@
         <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -7609,7 +7609,7 @@
         <v>0</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -7625,7 +7625,7 @@
         <v>0</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -7657,7 +7657,7 @@
         <v>0</v>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="48">
@@ -7673,7 +7673,7 @@
         <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -7689,7 +7689,7 @@
         <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -7737,7 +7737,7 @@
         <v>0</v>
       </c>
       <c r="D52" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -7753,7 +7753,7 @@
         <v>0</v>
       </c>
       <c r="D53" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -7769,7 +7769,7 @@
         <v>0</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="55">
@@ -7785,7 +7785,7 @@
         <v>0</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -7801,7 +7801,7 @@
         <v>0</v>
       </c>
       <c r="D56" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -7817,7 +7817,7 @@
         <v>0</v>
       </c>
       <c r="D57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -7833,7 +7833,7 @@
         <v>0</v>
       </c>
       <c r="D58" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -7849,7 +7849,7 @@
         <v>0</v>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="60">
@@ -7865,7 +7865,7 @@
         <v>0</v>
       </c>
       <c r="D60" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="61">
@@ -7881,7 +7881,7 @@
         <v>0</v>
       </c>
       <c r="D61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
@@ -7897,7 +7897,7 @@
         <v>0</v>
       </c>
       <c r="D62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -7913,7 +7913,7 @@
         <v>0</v>
       </c>
       <c r="D63" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="64">
@@ -7929,7 +7929,7 @@
         <v>0</v>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
@@ -7945,7 +7945,7 @@
         <v>0</v>
       </c>
       <c r="D65" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -7977,7 +7977,7 @@
         <v>0</v>
       </c>
       <c r="D67" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="68">
@@ -7993,7 +7993,7 @@
         <v>0</v>
       </c>
       <c r="D68" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="69">
@@ -8025,7 +8025,7 @@
         <v>0</v>
       </c>
       <c r="D70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -8041,7 +8041,7 @@
         <v>0</v>
       </c>
       <c r="D71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -8073,7 +8073,7 @@
         <v>0</v>
       </c>
       <c r="D73" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -8121,7 +8121,7 @@
         <v>0</v>
       </c>
       <c r="D76" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="77">
@@ -8137,7 +8137,7 @@
         <v>0</v>
       </c>
       <c r="D77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -8153,7 +8153,7 @@
         <v>0</v>
       </c>
       <c r="D78" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="79">
@@ -8185,7 +8185,7 @@
         <v>0</v>
       </c>
       <c r="D80" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81">
@@ -8201,7 +8201,7 @@
         <v>0</v>
       </c>
       <c r="D81" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -8217,7 +8217,7 @@
         <v>0</v>
       </c>
       <c r="D82" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -8233,7 +8233,7 @@
         <v>0</v>
       </c>
       <c r="D83" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -8249,7 +8249,7 @@
         <v>0</v>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="85">
@@ -8265,7 +8265,7 @@
         <v>0</v>
       </c>
       <c r="D85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -8313,7 +8313,7 @@
         <v>0</v>
       </c>
       <c r="D88" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89">
@@ -8329,7 +8329,7 @@
         <v>0</v>
       </c>
       <c r="D89" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="90">
@@ -8361,7 +8361,7 @@
         <v>0</v>
       </c>
       <c r="D91" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -8377,7 +8377,7 @@
         <v>0</v>
       </c>
       <c r="D92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -8393,7 +8393,7 @@
         <v>0</v>
       </c>
       <c r="D93" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="94">
@@ -8425,7 +8425,7 @@
         <v>0</v>
       </c>
       <c r="D95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96">
@@ -8441,7 +8441,7 @@
         <v>0</v>
       </c>
       <c r="D96" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -8473,7 +8473,7 @@
         <v>0</v>
       </c>
       <c r="D98" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -8537,7 +8537,7 @@
         <v>0</v>
       </c>
       <c r="D102" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="103">
@@ -8553,7 +8553,7 @@
         <v>0</v>
       </c>
       <c r="D103" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="104">
@@ -8569,7 +8569,7 @@
         <v>0</v>
       </c>
       <c r="D104" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105">
@@ -8585,7 +8585,7 @@
         <v>0</v>
       </c>
       <c r="D105" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
@@ -8601,7 +8601,7 @@
         <v>0</v>
       </c>
       <c r="D106" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107">
@@ -8617,7 +8617,7 @@
         <v>0</v>
       </c>
       <c r="D107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108">
@@ -8633,7 +8633,7 @@
         <v>0</v>
       </c>
       <c r="D108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109">
@@ -8649,7 +8649,7 @@
         <v>0</v>
       </c>
       <c r="D109" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110">
@@ -8681,7 +8681,7 @@
         <v>0</v>
       </c>
       <c r="D111" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112">
@@ -8697,7 +8697,7 @@
         <v>0</v>
       </c>
       <c r="D112" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="113">
@@ -8713,7 +8713,7 @@
         <v>0</v>
       </c>
       <c r="D113" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114">
@@ -8729,7 +8729,7 @@
         <v>0</v>
       </c>
       <c r="D114" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115">
@@ -8745,7 +8745,7 @@
         <v>0</v>
       </c>
       <c r="D115" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116">
@@ -8761,7 +8761,7 @@
         <v>0</v>
       </c>
       <c r="D116" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
@@ -8793,7 +8793,7 @@
         <v>0</v>
       </c>
       <c r="D118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119">
@@ -8809,7 +8809,7 @@
         <v>0</v>
       </c>
       <c r="D119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120">
@@ -8825,7 +8825,7 @@
         <v>0</v>
       </c>
       <c r="D120" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="121">
@@ -8857,7 +8857,7 @@
         <v>0</v>
       </c>
       <c r="D122" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="123">
@@ -8873,7 +8873,7 @@
         <v>0</v>
       </c>
       <c r="D123" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124">
@@ -8905,7 +8905,7 @@
         <v>0</v>
       </c>
       <c r="D125" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="126">
@@ -8921,7 +8921,7 @@
         <v>0</v>
       </c>
       <c r="D126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="127">
@@ -8953,7 +8953,7 @@
         <v>0</v>
       </c>
       <c r="D128" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129">
@@ -8969,7 +8969,7 @@
         <v>0</v>
       </c>
       <c r="D129" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130">
@@ -8985,7 +8985,7 @@
         <v>0</v>
       </c>
       <c r="D130" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="131">
@@ -9001,7 +9001,7 @@
         <v>0</v>
       </c>
       <c r="D131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132">
@@ -9017,7 +9017,7 @@
         <v>0</v>
       </c>
       <c r="D132" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="133">
@@ -9033,7 +9033,7 @@
         <v>0</v>
       </c>
       <c r="D133" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="134">
@@ -9049,7 +9049,7 @@
         <v>0</v>
       </c>
       <c r="D134" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="135">
@@ -9065,7 +9065,7 @@
         <v>0</v>
       </c>
       <c r="D135" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136">
@@ -9081,7 +9081,7 @@
         <v>0</v>
       </c>
       <c r="D136" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="137">
@@ -9113,7 +9113,7 @@
         <v>0</v>
       </c>
       <c r="D138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139">
@@ -9129,7 +9129,7 @@
         <v>0</v>
       </c>
       <c r="D139" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140">
@@ -9145,7 +9145,7 @@
         <v>0</v>
       </c>
       <c r="D140" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="141">
@@ -9161,7 +9161,7 @@
         <v>0</v>
       </c>
       <c r="D141" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="142">
@@ -9177,7 +9177,7 @@
         <v>0</v>
       </c>
       <c r="D142" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="143">
@@ -9193,7 +9193,7 @@
         <v>0</v>
       </c>
       <c r="D143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="144">
@@ -9209,7 +9209,7 @@
         <v>0</v>
       </c>
       <c r="D144" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="145">
@@ -9225,7 +9225,7 @@
         <v>0</v>
       </c>
       <c r="D145" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="146">
@@ -9241,7 +9241,7 @@
         <v>0</v>
       </c>
       <c r="D146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="147">
@@ -9257,7 +9257,7 @@
         <v>0</v>
       </c>
       <c r="D147" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="148">
@@ -9289,7 +9289,7 @@
         <v>0</v>
       </c>
       <c r="D149" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="150">
@@ -9321,7 +9321,7 @@
         <v>0</v>
       </c>
       <c r="D151" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152">
@@ -9337,7 +9337,7 @@
         <v>0</v>
       </c>
       <c r="D152" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="153">
@@ -9385,7 +9385,7 @@
         <v>0</v>
       </c>
       <c r="D155" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156">
@@ -9417,7 +9417,7 @@
         <v>0</v>
       </c>
       <c r="D157" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="158">
@@ -9449,7 +9449,7 @@
         <v>0</v>
       </c>
       <c r="D159" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160">
@@ -9481,7 +9481,7 @@
         <v>0</v>
       </c>
       <c r="D161" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="162">
@@ -9497,7 +9497,7 @@
         <v>0</v>
       </c>
       <c r="D162" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="163">
@@ -9513,7 +9513,7 @@
         <v>0</v>
       </c>
       <c r="D163" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="164">
@@ -9545,7 +9545,7 @@
         <v>0</v>
       </c>
       <c r="D165" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166">
@@ -9561,7 +9561,7 @@
         <v>0</v>
       </c>
       <c r="D166" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="167">
@@ -9577,7 +9577,7 @@
         <v>0</v>
       </c>
       <c r="D167" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168">
@@ -9641,7 +9641,7 @@
         <v>0</v>
       </c>
       <c r="D171" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="172">
@@ -9673,7 +9673,7 @@
         <v>0</v>
       </c>
       <c r="D173" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="174">
@@ -9689,7 +9689,7 @@
         <v>0</v>
       </c>
       <c r="D174" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="175">
@@ -9705,7 +9705,7 @@
         <v>0</v>
       </c>
       <c r="D175" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="176">
@@ -9721,7 +9721,7 @@
         <v>0</v>
       </c>
       <c r="D176" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177">
@@ -9737,7 +9737,7 @@
         <v>0</v>
       </c>
       <c r="D177" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="178">
@@ -9753,7 +9753,7 @@
         <v>0</v>
       </c>
       <c r="D178" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="179">
@@ -9769,7 +9769,7 @@
         <v>0</v>
       </c>
       <c r="D179" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="180">
@@ -9785,7 +9785,7 @@
         <v>0</v>
       </c>
       <c r="D180" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="181">
@@ -9817,7 +9817,7 @@
         <v>0</v>
       </c>
       <c r="D182" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="183">
@@ -9833,7 +9833,7 @@
         <v>0</v>
       </c>
       <c r="D183" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="184">
@@ -9849,7 +9849,7 @@
         <v>0</v>
       </c>
       <c r="D184" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="185">
@@ -9865,7 +9865,7 @@
         <v>0</v>
       </c>
       <c r="D185" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="186">
@@ -9881,7 +9881,7 @@
         <v>0</v>
       </c>
       <c r="D186" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="187">
@@ -9897,7 +9897,7 @@
         <v>0</v>
       </c>
       <c r="D187" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="188">
@@ -9929,7 +9929,7 @@
         <v>0</v>
       </c>
       <c r="D189" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="190">
@@ -9945,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="D190" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="191">
@@ -9961,7 +9961,7 @@
         <v>0</v>
       </c>
       <c r="D191" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="192">
@@ -9977,7 +9977,7 @@
         <v>0</v>
       </c>
       <c r="D192" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="193">
@@ -10009,7 +10009,7 @@
         <v>0</v>
       </c>
       <c r="D194" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="195">
@@ -10041,7 +10041,7 @@
         <v>0</v>
       </c>
       <c r="D196" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="197">
@@ -10057,7 +10057,7 @@
         <v>0</v>
       </c>
       <c r="D197" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="198">
@@ -10073,7 +10073,7 @@
         <v>0</v>
       </c>
       <c r="D198" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199">
@@ -10105,7 +10105,7 @@
         <v>0</v>
       </c>
       <c r="D200" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="201">
@@ -10121,7 +10121,7 @@
         <v>0</v>
       </c>
       <c r="D201" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>